<commit_message>
feat: finish second pass
</commit_message>
<xml_diff>
--- a/backend/measurements/corpus/scoring_pack/score_sheet1.xlsx
+++ b/backend/measurements/corpus/scoring_pack/score_sheet1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/randygyimah/Dev/em-fusion/backend/measurements/corpus/scoring_pack/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{81F25C90-1462-9045-8268-6997420BECCF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EE4C8C1E-978B-5348-9A58-15E35A981F0F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="20280" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -523,7 +523,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="224" uniqueCount="151">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="304" uniqueCount="151">
   <si>
     <t>Item</t>
   </si>
@@ -1415,8 +1415,12 @@
       <c r="H2" s="2">
         <v>3</v>
       </c>
-      <c r="I2" s="2"/>
-      <c r="J2" s="2"/>
+      <c r="I2" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="J2" s="2" t="s">
+        <v>102</v>
+      </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
@@ -1443,8 +1447,12 @@
       <c r="H3" s="2">
         <v>5</v>
       </c>
-      <c r="I3" s="2"/>
-      <c r="J3" s="2"/>
+      <c r="I3" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="J3" s="2" t="s">
+        <v>102</v>
+      </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
@@ -1471,8 +1479,12 @@
       <c r="H4" s="2">
         <v>5</v>
       </c>
-      <c r="I4" s="2"/>
-      <c r="J4" s="2"/>
+      <c r="I4" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="J4" s="2" t="s">
+        <v>103</v>
+      </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
@@ -1499,8 +1511,12 @@
       <c r="H5" s="2">
         <v>4</v>
       </c>
-      <c r="I5" s="2"/>
-      <c r="J5" s="2"/>
+      <c r="I5" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="J5" s="2" t="s">
+        <v>103</v>
+      </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
@@ -1527,8 +1543,12 @@
       <c r="H6" s="2">
         <v>3</v>
       </c>
-      <c r="I6" s="2"/>
-      <c r="J6" s="2"/>
+      <c r="I6" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="J6" s="2" t="s">
+        <v>102</v>
+      </c>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
@@ -1555,8 +1575,12 @@
       <c r="H7" s="2">
         <v>5</v>
       </c>
-      <c r="I7" s="2"/>
-      <c r="J7" s="2"/>
+      <c r="I7" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="J7" s="2" t="s">
+        <v>102</v>
+      </c>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
@@ -1583,8 +1607,12 @@
       <c r="H8" s="2">
         <v>5</v>
       </c>
-      <c r="I8" s="2"/>
-      <c r="J8" s="2"/>
+      <c r="I8" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="J8" s="2" t="s">
+        <v>102</v>
+      </c>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
@@ -1611,8 +1639,12 @@
       <c r="H9" s="2">
         <v>4</v>
       </c>
-      <c r="I9" s="2"/>
-      <c r="J9" s="2"/>
+      <c r="I9" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="J9" s="2" t="s">
+        <v>102</v>
+      </c>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
@@ -1639,8 +1671,12 @@
       <c r="H10" s="2">
         <v>4</v>
       </c>
-      <c r="I10" s="2"/>
-      <c r="J10" s="2"/>
+      <c r="I10" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="J10" s="2" t="s">
+        <v>102</v>
+      </c>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
@@ -1667,8 +1703,12 @@
       <c r="H11" s="2">
         <v>5</v>
       </c>
-      <c r="I11" s="2"/>
-      <c r="J11" s="2"/>
+      <c r="I11" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="J11" s="2" t="s">
+        <v>102</v>
+      </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
@@ -1695,8 +1735,12 @@
       <c r="H12" s="2">
         <v>5</v>
       </c>
-      <c r="I12" s="2"/>
-      <c r="J12" s="2"/>
+      <c r="I12" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="J12" s="2" t="s">
+        <v>102</v>
+      </c>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
@@ -1723,8 +1767,12 @@
       <c r="H13" s="2">
         <v>4</v>
       </c>
-      <c r="I13" s="2"/>
-      <c r="J13" s="2"/>
+      <c r="I13" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="J13" s="2" t="s">
+        <v>102</v>
+      </c>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
@@ -1751,8 +1799,12 @@
       <c r="H14" s="2">
         <v>4</v>
       </c>
-      <c r="I14" s="2"/>
-      <c r="J14" s="2"/>
+      <c r="I14" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="J14" s="2" t="s">
+        <v>102</v>
+      </c>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
@@ -1779,8 +1831,12 @@
       <c r="H15" s="2">
         <v>5</v>
       </c>
-      <c r="I15" s="2"/>
-      <c r="J15" s="2"/>
+      <c r="I15" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="J15" s="2" t="s">
+        <v>102</v>
+      </c>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
@@ -1807,8 +1863,12 @@
       <c r="H16" s="2">
         <v>5</v>
       </c>
-      <c r="I16" s="2"/>
-      <c r="J16" s="2"/>
+      <c r="I16" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="J16" s="2" t="s">
+        <v>102</v>
+      </c>
     </row>
     <row r="17" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
@@ -1835,8 +1895,12 @@
       <c r="H17" s="2">
         <v>4</v>
       </c>
-      <c r="I17" s="2"/>
-      <c r="J17" s="2"/>
+      <c r="I17" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="J17" s="2" t="s">
+        <v>102</v>
+      </c>
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
@@ -1863,8 +1927,12 @@
       <c r="H18" s="2">
         <v>5</v>
       </c>
-      <c r="I18" s="2"/>
-      <c r="J18" s="2"/>
+      <c r="I18" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="J18" s="2" t="s">
+        <v>102</v>
+      </c>
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
@@ -1891,8 +1959,12 @@
       <c r="H19" s="2">
         <v>3</v>
       </c>
-      <c r="I19" s="2"/>
-      <c r="J19" s="2"/>
+      <c r="I19" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="J19" s="2" t="s">
+        <v>102</v>
+      </c>
     </row>
     <row r="20" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
@@ -1919,8 +1991,12 @@
       <c r="H20" s="2">
         <v>3</v>
       </c>
-      <c r="I20" s="2"/>
-      <c r="J20" s="2"/>
+      <c r="I20" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="J20" s="2" t="s">
+        <v>102</v>
+      </c>
     </row>
     <row r="21" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
@@ -1947,8 +2023,12 @@
       <c r="H21" s="2">
         <v>5</v>
       </c>
-      <c r="I21" s="2"/>
-      <c r="J21" s="2"/>
+      <c r="I21" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="J21" s="2" t="s">
+        <v>102</v>
+      </c>
     </row>
     <row r="22" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
@@ -1975,8 +2055,12 @@
       <c r="H22" s="2">
         <v>5</v>
       </c>
-      <c r="I22" s="2"/>
-      <c r="J22" s="2"/>
+      <c r="I22" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="J22" s="2" t="s">
+        <v>103</v>
+      </c>
     </row>
     <row r="23" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
@@ -2003,8 +2087,12 @@
       <c r="H23" s="2">
         <v>4</v>
       </c>
-      <c r="I23" s="2"/>
-      <c r="J23" s="2"/>
+      <c r="I23" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="J23" s="2" t="s">
+        <v>103</v>
+      </c>
     </row>
     <row r="24" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
@@ -2031,8 +2119,12 @@
       <c r="H24" s="2">
         <v>4</v>
       </c>
-      <c r="I24" s="2"/>
-      <c r="J24" s="2"/>
+      <c r="I24" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="J24" s="2" t="s">
+        <v>103</v>
+      </c>
     </row>
     <row r="25" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
@@ -2059,8 +2151,12 @@
       <c r="H25" s="2">
         <v>5</v>
       </c>
-      <c r="I25" s="2"/>
-      <c r="J25" s="2"/>
+      <c r="I25" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="J25" s="2" t="s">
+        <v>103</v>
+      </c>
     </row>
     <row r="26" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
@@ -2087,8 +2183,12 @@
       <c r="H26" s="2">
         <v>4</v>
       </c>
-      <c r="I26" s="2"/>
-      <c r="J26" s="2"/>
+      <c r="I26" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="J26" s="2" t="s">
+        <v>103</v>
+      </c>
     </row>
     <row r="27" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
@@ -2115,8 +2215,12 @@
       <c r="H27" s="2">
         <v>5</v>
       </c>
-      <c r="I27" s="2"/>
-      <c r="J27" s="2"/>
+      <c r="I27" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="J27" s="2" t="s">
+        <v>103</v>
+      </c>
     </row>
     <row r="28" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
@@ -2143,8 +2247,12 @@
       <c r="H28" s="2">
         <v>5</v>
       </c>
-      <c r="I28" s="2"/>
-      <c r="J28" s="2"/>
+      <c r="I28" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="J28" s="2" t="s">
+        <v>103</v>
+      </c>
     </row>
     <row r="29" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
@@ -2171,8 +2279,12 @@
       <c r="H29" s="2">
         <v>4</v>
       </c>
-      <c r="I29" s="2"/>
-      <c r="J29" s="2"/>
+      <c r="I29" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="J29" s="2" t="s">
+        <v>103</v>
+      </c>
     </row>
     <row r="30" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
@@ -2199,8 +2311,12 @@
       <c r="H30" s="2">
         <v>5</v>
       </c>
-      <c r="I30" s="2"/>
-      <c r="J30" s="2"/>
+      <c r="I30" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="J30" s="2" t="s">
+        <v>103</v>
+      </c>
     </row>
     <row r="31" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
@@ -2227,8 +2343,12 @@
       <c r="H31" s="2">
         <v>4</v>
       </c>
-      <c r="I31" s="2"/>
-      <c r="J31" s="2"/>
+      <c r="I31" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="J31" s="2" t="s">
+        <v>103</v>
+      </c>
     </row>
     <row r="32" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
@@ -2255,8 +2375,12 @@
       <c r="H32" s="2">
         <v>4</v>
       </c>
-      <c r="I32" s="2"/>
-      <c r="J32" s="2"/>
+      <c r="I32" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="J32" s="2" t="s">
+        <v>104</v>
+      </c>
     </row>
     <row r="33" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
@@ -2283,8 +2407,12 @@
       <c r="H33" s="2">
         <v>5</v>
       </c>
-      <c r="I33" s="2"/>
-      <c r="J33" s="2"/>
+      <c r="I33" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="J33" s="2" t="s">
+        <v>104</v>
+      </c>
     </row>
     <row r="34" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
@@ -2311,8 +2439,12 @@
       <c r="H34" s="2">
         <v>4</v>
       </c>
-      <c r="I34" s="2"/>
-      <c r="J34" s="2"/>
+      <c r="I34" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="J34" s="2" t="s">
+        <v>104</v>
+      </c>
     </row>
     <row r="35" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
@@ -2339,8 +2471,12 @@
       <c r="H35" s="2">
         <v>5</v>
       </c>
-      <c r="I35" s="2"/>
-      <c r="J35" s="2"/>
+      <c r="I35" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="J35" s="2" t="s">
+        <v>104</v>
+      </c>
     </row>
     <row r="36" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
@@ -2367,8 +2503,12 @@
       <c r="H36" s="2">
         <v>4</v>
       </c>
-      <c r="I36" s="2"/>
-      <c r="J36" s="2"/>
+      <c r="I36" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="J36" s="2" t="s">
+        <v>104</v>
+      </c>
     </row>
     <row r="37" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
@@ -2395,8 +2535,12 @@
       <c r="H37" s="2">
         <v>5</v>
       </c>
-      <c r="I37" s="2"/>
-      <c r="J37" s="2"/>
+      <c r="I37" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="J37" s="2" t="s">
+        <v>104</v>
+      </c>
     </row>
     <row r="38" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
@@ -2423,8 +2567,12 @@
       <c r="H38" s="2">
         <v>4</v>
       </c>
-      <c r="I38" s="2"/>
-      <c r="J38" s="2"/>
+      <c r="I38" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="J38" s="2" t="s">
+        <v>104</v>
+      </c>
     </row>
     <row r="39" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
@@ -2451,8 +2599,12 @@
       <c r="H39" s="2">
         <v>5</v>
       </c>
-      <c r="I39" s="2"/>
-      <c r="J39" s="2"/>
+      <c r="I39" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="J39" s="2" t="s">
+        <v>104</v>
+      </c>
     </row>
     <row r="40" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
@@ -2479,8 +2631,12 @@
       <c r="H40" s="2">
         <v>4</v>
       </c>
-      <c r="I40" s="2"/>
-      <c r="J40" s="2"/>
+      <c r="I40" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="J40" s="2" t="s">
+        <v>104</v>
+      </c>
     </row>
     <row r="41" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
@@ -2507,8 +2663,12 @@
       <c r="H41" s="2">
         <v>5</v>
       </c>
-      <c r="I41" s="2"/>
-      <c r="J41" s="2"/>
+      <c r="I41" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="J41" s="2" t="s">
+        <v>104</v>
+      </c>
     </row>
   </sheetData>
   <sheetProtection sheet="1"/>

</xml_diff>